<commit_message>
Add additional ablation experiments and final report update
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1379,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AG61"/>
+  <dimension ref="A1:AG65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="19" min="1" max="1"/>
@@ -4691,6 +4691,399 @@
         <f>IF(OR(AF61="",Seeds!$C$10=""),"",IF(ABS(AF61)&gt;Seeds!$C$10,"Có","Không"))</f>
         <v/>
       </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="19" t="inlineStr">
+        <is>
+          <t>amp-bf16</t>
+        </is>
+      </c>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>amp</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>CPU bf16 autocast</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="inlineStr">
+        <is>
+          <t>adam</t>
+        </is>
+      </c>
+      <c r="F62" s="19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="19" t="n">
+        <v>512</v>
+      </c>
+      <c r="I62" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J62" s="19" t="inlineStr">
+        <is>
+          <t>[256, 128]</t>
+        </is>
+      </c>
+      <c r="K62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M62" s="19" t="inlineStr">
+        <is>
+          <t>bf16</t>
+        </is>
+      </c>
+      <c r="N62" s="19" t="inlineStr">
+        <is>
+          <t>he</t>
+        </is>
+      </c>
+      <c r="O62" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="P62" s="19" t="n">
+        <v>2.310553499672654</v>
+      </c>
+      <c r="Q62" s="19" t="n">
+        <v>0.2368694463685571</v>
+      </c>
+      <c r="R62" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="S62" s="19" t="n">
+        <v>0.2150714142370224</v>
+      </c>
+      <c r="T62" s="19" t="n">
+        <v>0.2368694463685571</v>
+      </c>
+      <c r="U62" s="19" t="n">
+        <v>0.9057787052774252</v>
+      </c>
+      <c r="V62" s="19" t="n">
+        <v>0.8466016709959095</v>
+      </c>
+      <c r="W62" s="19" t="n">
+        <v>3.601837590001378</v>
+      </c>
+      <c r="X62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y62" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB62" s="19" t="inlineStr">
+        <is>
+          <t>figures/amp-bf16.png</t>
+        </is>
+      </c>
+      <c r="AC62" s="19" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="19" t="inlineStr">
+        <is>
+          <t>hparam-adamw</t>
+        </is>
+      </c>
+      <c r="B63" s="19" t="inlineStr">
+        <is>
+          <t>hparam</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>AdamW + weight decay</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="E63" s="19" t="inlineStr">
+        <is>
+          <t>adamw</t>
+        </is>
+      </c>
+      <c r="F63" s="19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G63" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H63" s="19" t="n">
+        <v>512</v>
+      </c>
+      <c r="I63" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J63" s="19" t="inlineStr">
+        <is>
+          <t>[256, 128]</t>
+        </is>
+      </c>
+      <c r="K63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" s="19" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="N63" s="19" t="inlineStr">
+        <is>
+          <t>he</t>
+        </is>
+      </c>
+      <c r="O63" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="P63" s="19" t="n">
+        <v>1.900539940096667</v>
+      </c>
+      <c r="Q63" s="19" t="n">
+        <v>0.2414391803540384</v>
+      </c>
+      <c r="R63" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="S63" s="19" t="n">
+        <v>0.22954156291008</v>
+      </c>
+      <c r="T63" s="19" t="n">
+        <v>0.24853127553188</v>
+      </c>
+      <c r="U63" s="19" t="n">
+        <v>0.9011316451883565</v>
+      </c>
+      <c r="V63" s="19" t="n">
+        <v>0.8485659534191904</v>
+      </c>
+      <c r="W63" s="19" t="n">
+        <v>1.911763685001642</v>
+      </c>
+      <c r="X63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y63" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z63" t="n">
+        <v>0.9026</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>0.8531</v>
+      </c>
+      <c r="AB63" s="19" t="inlineStr">
+        <is>
+          <t>figures/hparam-adamw.png</t>
+        </is>
+      </c>
+      <c r="AC63" s="19" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="19" t="inlineStr">
+        <is>
+          <t>init-xavier</t>
+        </is>
+      </c>
+      <c r="B64" s="19" t="inlineStr">
+        <is>
+          <t>init</t>
+        </is>
+      </c>
+      <c r="C64" s="19" t="inlineStr">
+        <is>
+          <t>Xavier init with Adam</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="E64" s="19" t="inlineStr">
+        <is>
+          <t>adam</t>
+        </is>
+      </c>
+      <c r="F64" s="19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="19" t="n">
+        <v>512</v>
+      </c>
+      <c r="I64" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J64" s="19" t="inlineStr">
+        <is>
+          <t>[256, 128]</t>
+        </is>
+      </c>
+      <c r="K64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" s="19" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="N64" s="19" t="inlineStr">
+        <is>
+          <t>xavier</t>
+        </is>
+      </c>
+      <c r="O64" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="P64" s="19" t="n">
+        <v>1.985815929083146</v>
+      </c>
+      <c r="Q64" s="19" t="n">
+        <v>0.2494165387047653</v>
+      </c>
+      <c r="R64" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="S64" s="19" t="n">
+        <v>0.2319661612319946</v>
+      </c>
+      <c r="T64" s="19" t="n">
+        <v>0.2494165387047653</v>
+      </c>
+      <c r="U64" s="19" t="n">
+        <v>0.9002388072545772</v>
+      </c>
+      <c r="V64" s="19" t="n">
+        <v>0.846246698090563</v>
+      </c>
+      <c r="W64" s="19" t="n">
+        <v>1.995254000000568</v>
+      </c>
+      <c r="X64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y64" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB64" s="19" t="inlineStr">
+        <is>
+          <t>figures/init-xavier.png</t>
+        </is>
+      </c>
+      <c r="AC64" s="19" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="19" t="inlineStr">
+        <is>
+          <t>loss-mse</t>
+        </is>
+      </c>
+      <c r="B65" s="19" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="C65" s="19" t="inlineStr">
+        <is>
+          <t>MSE loss with Adam</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="inlineStr">
+        <is>
+          <t>mse</t>
+        </is>
+      </c>
+      <c r="E65" s="19" t="inlineStr">
+        <is>
+          <t>adam</t>
+        </is>
+      </c>
+      <c r="F65" s="19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="19" t="n">
+        <v>512</v>
+      </c>
+      <c r="I65" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J65" s="19" t="inlineStr">
+        <is>
+          <t>[256, 128]</t>
+        </is>
+      </c>
+      <c r="K65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" s="19" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="N65" s="19" t="inlineStr">
+        <is>
+          <t>he</t>
+        </is>
+      </c>
+      <c r="O65" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="P65" s="19" t="n">
+        <v>0.3967943757061386</v>
+      </c>
+      <c r="Q65" s="19" t="n">
+        <v>0.02320597477649809</v>
+      </c>
+      <c r="R65" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="S65" s="19" t="n">
+        <v>0.02181514468789101</v>
+      </c>
+      <c r="T65" s="19" t="n">
+        <v>0.02320597477649809</v>
+      </c>
+      <c r="U65" s="19" t="n">
+        <v>0.9031970052279426</v>
+      </c>
+      <c r="V65" s="19" t="n">
+        <v>0.8338605089426052</v>
+      </c>
+      <c r="W65" s="19" t="n">
+        <v>1.785585939999146</v>
+      </c>
+      <c r="X65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y65" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB65" s="19" t="inlineStr">
+        <is>
+          <t>figures/loss-mse.png</t>
+        </is>
+      </c>
+      <c r="AC65" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AG61"/>

</xml_diff>